<commit_message>
FEAT: uploaded survey results + corrected an error in survey one candidate (1 multi-hop flag wrong)
</commit_message>
<xml_diff>
--- a/phase_1_validation/human_validation/survey_candidate_1.xlsx
+++ b/phase_1_validation/human_validation/survey_candidate_1.xlsx
@@ -948,7 +948,7 @@
       </c>
       <c r="Q4" s="1" t="n">
         <f aca="false">AVERAGE(G2:G151)</f>
-        <v>0.756756756756757</v>
+        <v>0.72972972972973</v>
       </c>
       <c r="R4" s="1" t="n">
         <f aca="false">AVERAGE(H2:H151)</f>
@@ -977,7 +977,7 @@
       <c r="K5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L5" s="0" t="n">
+      <c r="L5" s="1" t="n">
         <f aca="false">SUMPRODUCT((MOD(ROW(D2:D151)-ROW(D2),6)=0)*D2:D151)/SUMPRODUCT(--(MOD(ROW(D2:D151)-ROW(D2),6)=0))</f>
         <v>0.84</v>
       </c>
@@ -985,11 +985,10 @@
         <f aca="false">SUMPRODUCT((MOD(ROW(E2:E151)-ROW(E2),6)=0)*E2:E151)/SUMPRODUCT(--(MOD(ROW(E2:E151)-ROW(E2),6)=0))</f>
         <v>0.88</v>
       </c>
-      <c r="N5" s="0" t="n">
+      <c r="N5" s="1" t="n">
         <f aca="false">SUMPRODUCT((MOD(ROW(F2:F151)-ROW(F2),6)=0)*F2:F151)/SUMPRODUCT(--(MOD(ROW(F2:F151)-ROW(F2),6)=0))</f>
         <v>0.96</v>
       </c>
-      <c r="O5" s="0"/>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4"/>
@@ -1017,7 +1016,7 @@
       <c r="K6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="L6" s="0" t="n">
+      <c r="L6" s="1" t="n">
         <f aca="false">SUMPRODUCT((MOD(ROW(D3:D152)-ROW(D3),6)=0)*D3:D152)/SUMPRODUCT(--(MOD(ROW(D3:D152)-ROW(D3),6)=0))</f>
         <v>0.8</v>
       </c>
@@ -1025,11 +1024,11 @@
         <f aca="false">SUMPRODUCT((MOD(ROW(E3:E152)-ROW(E3),6)=0)*E3:E152)/SUMPRODUCT(--(MOD(ROW(E3:E152)-ROW(E3),6)=0))</f>
         <v>0.84</v>
       </c>
-      <c r="N6" s="0" t="n">
+      <c r="N6" s="1" t="n">
         <f aca="false">SUMPRODUCT((MOD(ROW(F3:F152)-ROW(F3),6)=0)*F3:F152)/SUMPRODUCT(--(MOD(ROW(F3:F152)-ROW(F3),6)=0))</f>
         <v>0.92</v>
       </c>
-      <c r="R6" s="0" t="n">
+      <c r="R6" s="1" t="n">
         <f aca="false">SUMPRODUCT((MOD(ROW(H3:H151)-ROW(H3),6)=0)*(H3:H151&lt;&gt;"")*H3:H151)/SUMPRODUCT((MOD(ROW(H3:H151)-ROW(H3),6)=0)*(H3:H151&lt;&gt;""))</f>
         <v>0.9</v>
       </c>
@@ -1062,7 +1061,7 @@
       <c r="K7" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="L7" s="0" t="n">
+      <c r="L7" s="1" t="n">
         <f aca="false">SUMPRODUCT((MOD(ROW(D4:D153)-ROW(D4),6)=0)*D4:D153)/SUMPRODUCT(--(MOD(ROW(D4:D153)-ROW(D4),6)=0))</f>
         <v>0.92</v>
       </c>
@@ -1070,11 +1069,11 @@
         <f aca="false">SUMPRODUCT((MOD(ROW(E4:E153)-ROW(E4),6)=0)*E4:E153)/SUMPRODUCT(--(MOD(ROW(E4:E153)-ROW(E4),6)=0))</f>
         <v>0.84</v>
       </c>
-      <c r="N7" s="0" t="n">
+      <c r="N7" s="1" t="n">
         <f aca="false">SUMPRODUCT((MOD(ROW(F4:F153)-ROW(F4),6)=0)*F4:F153)/SUMPRODUCT(--(MOD(ROW(F4:F153)-ROW(F4),6)=0))</f>
         <v>0.92</v>
       </c>
-      <c r="R7" s="0" t="n">
+      <c r="R7" s="1" t="n">
         <f aca="false">SUMPRODUCT((MOD(ROW(H4:H152)-ROW(H4),5)=0)*(H4:H152&lt;&gt;"")*H4:H152)/SUMPRODUCT((MOD(ROW(H4:H152)-ROW(H4),5)=0)*(H4:H152&lt;&gt;""))</f>
         <v>0.8</v>
       </c>
@@ -1103,7 +1102,7 @@
       <c r="K8" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L8" s="0" t="n">
+      <c r="L8" s="1" t="n">
         <f aca="false">SUMPRODUCT((MOD(ROW(D5:D154)-ROW(D5),6)=0)*D5:D154)/SUMPRODUCT(--(MOD(ROW(D5:D154)-ROW(D5),6)=0))</f>
         <v>0.68</v>
       </c>
@@ -1111,7 +1110,7 @@
         <f aca="false">SUMPRODUCT((MOD(ROW(E5:E154)-ROW(E5),6)=0)*E5:E154)/SUMPRODUCT(--(MOD(ROW(E5:E154)-ROW(E5),6)=0))</f>
         <v>0.84</v>
       </c>
-      <c r="N8" s="0" t="n">
+      <c r="N8" s="1" t="n">
         <f aca="false">SUMPRODUCT((MOD(ROW(F5:F154)-ROW(F5),6)=0)*F5:F154)/SUMPRODUCT(--(MOD(ROW(F5:F154)-ROW(F5),6)=0))</f>
         <v>0.96</v>
       </c>
@@ -1140,7 +1139,7 @@
       <c r="K9" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="L9" s="0" t="n">
+      <c r="L9" s="1" t="n">
         <f aca="false">SUMPRODUCT((MOD(ROW(D6:D155)-ROW(D6),6)=0)*D6:D155)/SUMPRODUCT(--(MOD(ROW(D6:D155)-ROW(D6),6)=0))</f>
         <v>0.76</v>
       </c>
@@ -1148,7 +1147,7 @@
         <f aca="false">SUMPRODUCT((MOD(ROW(E6:E155)-ROW(E6),6)=0)*E6:E155)/SUMPRODUCT(--(MOD(ROW(E6:E155)-ROW(E6),6)=0))</f>
         <v>0.8</v>
       </c>
-      <c r="N9" s="0" t="n">
+      <c r="N9" s="1" t="n">
         <f aca="false">SUMPRODUCT((MOD(ROW(F6:F155)-ROW(F6),6)=0)*F6:F155)/SUMPRODUCT(--(MOD(ROW(F6:F155)-ROW(F6),6)=0))</f>
         <v>0.92</v>
       </c>
@@ -3999,7 +3998,7 @@
         <v>1</v>
       </c>
       <c r="G132" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H132" s="11"/>
       <c r="I132" s="11"/>

</xml_diff>